<commit_message>
Subo estrucuta abacus y arreglo ejercicio 1 abacus
</commit_message>
<xml_diff>
--- a/abacus/ejercicio1Abacus.xlsx
+++ b/abacus/ejercicio1Abacus.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ignacio\Desktop\Archivos\VirtualMachine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99C336B0-5E44-48A1-9D1C-5FB6FC1CF4C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{91B57320-4587-4706-924E-924B5579FD0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="70">
   <si>
     <t>Estrategia:</t>
   </si>
@@ -142,12 +142,6 @@
   </si>
   <si>
     <t>4- Si es distinto, avanzar de posicion (bifurcar</t>
-  </si>
-  <si>
-    <t>8XXX</t>
-  </si>
-  <si>
-    <t>9XXX</t>
   </si>
   <si>
     <t>Si es igual, cargamos en vector</t>
@@ -882,7 +876,7 @@
     </row>
     <row r="48" spans="2:3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B48" s="35" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C48" s="35"/>
     </row>
@@ -982,7 +976,7 @@
         <v>2</v>
       </c>
       <c r="C59" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -1117,32 +1111,32 @@
         <v>21</v>
       </c>
       <c r="B72" s="17" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C72" s="15" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B73" s="20" t="s">
-        <v>39</v>
+      <c r="B73" s="20">
+        <v>8319</v>
       </c>
       <c r="C73" s="18" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="B74" s="20" t="s">
+      <c r="B74" s="20">
+        <v>9319</v>
+      </c>
+      <c r="C74" s="18" t="s">
         <v>40</v>
-      </c>
-      <c r="C74" s="18" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
@@ -1153,7 +1147,7 @@
         <v>1401</v>
       </c>
       <c r="C75" s="21" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
@@ -1164,7 +1158,7 @@
         <v>3251</v>
       </c>
       <c r="C76" s="21" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
@@ -1175,7 +1169,7 @@
         <v>2401</v>
       </c>
       <c r="C77" s="21" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
@@ -1186,7 +1180,7 @@
         <v>1309</v>
       </c>
       <c r="C78" s="23" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
@@ -1197,7 +1191,7 @@
         <v>3251</v>
       </c>
       <c r="C79" s="23" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
@@ -1208,7 +1202,7 @@
         <v>2314</v>
       </c>
       <c r="C80" s="23" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
@@ -1219,7 +1213,7 @@
         <v>14</v>
       </c>
       <c r="C81" s="23" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
@@ -1230,7 +1224,7 @@
         <v>2100</v>
       </c>
       <c r="C82" s="27" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
@@ -1241,7 +1235,7 @@
         <v>1315</v>
       </c>
       <c r="C83" s="27" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
@@ -1252,7 +1246,7 @@
         <v>3251</v>
       </c>
       <c r="C84" s="27" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
@@ -1263,7 +1257,7 @@
         <v>2315</v>
       </c>
       <c r="C85" s="27" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
@@ -1274,73 +1268,73 @@
         <v>1309</v>
       </c>
       <c r="C86" s="30" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="31" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B87" s="32">
-        <v>3252</v>
+        <v>3253</v>
       </c>
       <c r="C87" s="30" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="31" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B88" s="32" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C88" s="30" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="31" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B89" s="32" t="s">
         <v>14</v>
       </c>
       <c r="C89" s="30" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="31" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B90" s="32">
         <v>2200</v>
       </c>
       <c r="C90" s="30" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="33" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B91" s="34">
         <v>7306</v>
       </c>
       <c r="C91" s="35" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="33" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B92" s="34">
         <v>8306</v>
       </c>
       <c r="C92" s="35" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
@@ -1348,10 +1342,10 @@
         <v>320</v>
       </c>
       <c r="B93" s="37" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C93" s="38" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>